<commit_message>
[IMP] flags customer and supplier
</commit_message>
<xml_diff>
--- a/clodoo/transodoo.xlsx
+++ b/clodoo/transodoo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="859">
   <si>
     <t xml:space="preserve">model</t>
   </si>
@@ -2519,6 +2519,18 @@
   </si>
   <si>
     <t xml:space="preserve">zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_supplier</t>
   </si>
   <si>
     <t xml:space="preserve">res.users</t>
@@ -11058,35 +11070,37 @@
     </row>
     <row r="539" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A539" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B539" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D539" s="1" t="s">
         <v>833</v>
       </c>
-      <c r="B539" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D539" s="1" t="s">
+      <c r="E539" s="3"/>
+      <c r="M539" s="1" t="s">
         <v>834</v>
-      </c>
-      <c r="E539" s="3" t="s">
-        <v>835</v>
       </c>
     </row>
     <row r="540" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A540" s="3" t="s">
-        <v>833</v>
+        <v>192</v>
       </c>
       <c r="B540" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D540" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="E540" s="3"/>
+      <c r="M540" s="1" t="s">
         <v>836</v>
-      </c>
-      <c r="E540" s="3" t="s">
-        <v>837</v>
       </c>
     </row>
     <row r="541" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A541" s="3" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B541" s="3" t="s">
         <v>27</v>
@@ -11100,85 +11114,85 @@
     </row>
     <row r="542" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A542" s="3" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B542" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="D542" s="1" t="s">
+        <v>840</v>
+      </c>
       <c r="E542" s="3" t="s">
-        <v>826</v>
+        <v>841</v>
       </c>
     </row>
     <row r="543" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A543" s="3" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B543" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="D543" s="1" t="s">
+        <v>842</v>
+      </c>
       <c r="E543" s="3" t="s">
-        <v>93</v>
+        <v>843</v>
       </c>
     </row>
     <row r="544" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A544" s="3" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B544" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D544" s="1" t="s">
-        <v>841</v>
-      </c>
-      <c r="G544" s="3" t="s">
-        <v>842</v>
+        <v>27</v>
+      </c>
+      <c r="E544" s="3" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="545" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A545" s="3" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B545" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D545" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="H545" s="1" t="s">
-        <v>132</v>
+      <c r="E545" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="546" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A546" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B546" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C546" s="1" t="s">
-        <v>163</v>
+        <v>111</v>
       </c>
       <c r="D546" s="1" t="s">
-        <v>719</v>
+        <v>845</v>
+      </c>
+      <c r="G546" s="3" t="s">
+        <v>846</v>
       </c>
     </row>
     <row r="547" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A547" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B547" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C547" s="1" t="s">
-        <v>163</v>
+        <v>27</v>
       </c>
       <c r="D547" s="1" t="s">
-        <v>739</v>
+        <v>131</v>
+      </c>
+      <c r="H547" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="548" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A548" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B548" s="3" t="s">
         <v>33</v>
@@ -11187,12 +11201,12 @@
         <v>163</v>
       </c>
       <c r="D548" s="1" t="s">
-        <v>736</v>
+        <v>719</v>
       </c>
     </row>
     <row r="549" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A549" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B549" s="3" t="s">
         <v>33</v>
@@ -11201,15 +11215,12 @@
         <v>163</v>
       </c>
       <c r="D549" s="1" t="s">
-        <v>843</v>
-      </c>
-      <c r="G549" s="3" t="s">
-        <v>144</v>
+        <v>739</v>
       </c>
     </row>
     <row r="550" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A550" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B550" s="3" t="s">
         <v>33</v>
@@ -11218,15 +11229,12 @@
         <v>163</v>
       </c>
       <c r="D550" s="1" t="s">
-        <v>844</v>
-      </c>
-      <c r="G550" s="3" t="s">
-        <v>144</v>
+        <v>736</v>
       </c>
     </row>
     <row r="551" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A551" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B551" s="3" t="s">
         <v>33</v>
@@ -11235,7 +11243,7 @@
         <v>163</v>
       </c>
       <c r="D551" s="1" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="G551" s="3" t="s">
         <v>144</v>
@@ -11243,7 +11251,7 @@
     </row>
     <row r="552" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A552" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B552" s="3" t="s">
         <v>33</v>
@@ -11252,12 +11260,15 @@
         <v>163</v>
       </c>
       <c r="D552" s="1" t="s">
-        <v>742</v>
+        <v>848</v>
+      </c>
+      <c r="G552" s="3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="553" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A553" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B553" s="3" t="s">
         <v>33</v>
@@ -11266,7 +11277,7 @@
         <v>163</v>
       </c>
       <c r="D553" s="1" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="G553" s="3" t="s">
         <v>144</v>
@@ -11274,7 +11285,7 @@
     </row>
     <row r="554" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A554" s="3" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="B554" s="3" t="s">
         <v>33</v>
@@ -11283,26 +11294,29 @@
         <v>163</v>
       </c>
       <c r="D554" s="1" t="s">
-        <v>847</v>
-      </c>
-      <c r="G554" s="3" t="s">
-        <v>144</v>
+        <v>742</v>
       </c>
     </row>
     <row r="555" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A555" s="3" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
       <c r="B555" s="3" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="C555" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="D555" s="1" t="s">
-        <v>849</v>
+        <v>850</v>
+      </c>
+      <c r="G555" s="3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="556" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A556" s="3" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
       <c r="B556" s="3" t="s">
         <v>33</v>
@@ -11311,29 +11325,26 @@
         <v>163</v>
       </c>
       <c r="D556" s="1" t="s">
-        <v>719</v>
+        <v>851</v>
+      </c>
+      <c r="G556" s="3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="557" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A557" s="3" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="B557" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C557" s="1" t="s">
-        <v>163</v>
+        <v>27</v>
       </c>
       <c r="D557" s="1" t="s">
-        <v>737</v>
-      </c>
-      <c r="H557" s="1" t="s">
-        <v>144</v>
+        <v>853</v>
       </c>
     </row>
     <row r="558" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A558" s="3" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="B558" s="3" t="s">
         <v>33</v>
@@ -11342,12 +11353,12 @@
         <v>163</v>
       </c>
       <c r="D558" s="1" t="s">
-        <v>739</v>
+        <v>719</v>
       </c>
     </row>
     <row r="559" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A559" s="3" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="B559" s="3" t="s">
         <v>33</v>
@@ -11356,12 +11367,15 @@
         <v>163</v>
       </c>
       <c r="D559" s="1" t="s">
-        <v>736</v>
+        <v>737</v>
+      </c>
+      <c r="H559" s="1" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="560" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A560" s="3" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="B560" s="3" t="s">
         <v>33</v>
@@ -11370,50 +11384,76 @@
         <v>163</v>
       </c>
       <c r="D560" s="1" t="s">
-        <v>850</v>
-      </c>
-      <c r="H560" s="1" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
     </row>
     <row r="561" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A561" s="3" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B561" s="3" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="C561" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="D561" s="1" t="s">
-        <v>852</v>
+        <v>736</v>
       </c>
     </row>
     <row r="562" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A562" s="3" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B562" s="3" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="C562" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="D562" s="1" t="s">
-        <v>136</v>
+        <v>854</v>
+      </c>
+      <c r="H562" s="1" t="s">
+        <v>736</v>
       </c>
     </row>
     <row r="563" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A563" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B563" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D563" s="1" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="564" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A564" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="B564" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D564" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="565" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A565" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="B565" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D565" s="1" t="s">
         <v>617</v>
       </c>
-      <c r="G563" s="3" t="s">
+      <c r="G565" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>